<commit_message>
Auto: Week 34/2026 data extracted from PDFs
</commit_message>
<xml_diff>
--- a/Gulf_Dashboard_W34_2026.xlsx
+++ b/Gulf_Dashboard_W34_2026.xlsx
@@ -779,52 +779,29 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t> 1.Delay of SAO bridge and box convert construction ( 3 bridges and 2 box culverts)
-Box culvert STA. 1+434 (West RW07) Box culvert STA. 2+704 (West RW01)
-Bridge STA.2+950 (East RW17) Bridge STA.3+750 (West RW01)
-Bridge STA.4+491 (East RW17)
- 2.Low production rate of rebar installation
-- WTG11 Rebar binding 74 Days
-- WTG12 Rebar binding 63 Days
-- WTG14 Rebar binding 67 Days
-- WTG04 Rebar binding 45 Days
-Based on the current site arrangement, there is a drainage concern related to the Box Culvert area
-at East Side RW17 Sta 0+500, which may be affect to the equipment/material laydown arrangement
-from Silamas.
-Box culvert
- 1.Request cooperation from Chief Executive of the
-Non sawang SAO incase stagnant water from road
-project. (Box culvert completed)
- 2.Unofficial Environmental &amp; Social Complaints
-Local residents are complaining about stagnant water from
-road project
-- West side 2 person (Box culvert completed)</t>
-        </is>
-      </c>
+      <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Clearing and grubbing RW1,RW2
-2Continue Box culvert RW17 STA 0+500,1+845
-Backfilling
-V ditch RW17
-- East : RW03
--East : RW9,RW15
-- East : RW17 STA 4+600 to 5+300
-- East : RW17 3+500 to 4+000
-Rebar binding and formwork installation WTG11,WTG12,WTG04,WTG15,WTG07
-Soil improvement WTG16,WTG17
-Concrete foundation WTG12
-Repairing and baclfilling WTG05,WTG13,WTG08,WTG6
-Cable pulling feeder 1 RW07,RW01
-Continue duct bank RW3,RW10
-• Backfilling RCP RW6 21
-Grouting vertical joint 3 rings
-Assembly of concrete ring 3 rings
-Quarter ring delivery 36 ea
-Substation control building
-- Masonry block ground floor</t>
+          <t>[BOP(STECON)] Clearing and grubbing RW1,RW9
+[BOP(STECON)] Selected A RW9,RW15
+[BOP(STECON)] Subbase,Crushrock RW17
+[BOP(STECON)] Rebar,FWinstallation WTG4,WTG11,WTG12,WTG14,WTG15
+[BOP(STECON)] Repairing,Backfilling WTG5,WTG13,WTG8
+[BOP(STECON)] Concrete cover casting WTG8,WTG13
+[BOP(STECON)] Concrete pole installation RW17,RW7
+[BOP(STECON)] Cable pulling feeder 1
+[BOP(STECON)] Remove formwork WTG6
+[TSA (GOLDWIND)] Assembly of quarter ring segment 3 rings
+[TSA (GOLDWIND)] Grouting vertical joint 3 rings
+[Plant Substation(SIEMENS)] Roof slab concrete casting and ground floor masonry work(Control building)
+[Plant Substation(SIEMENS)] Wall SWYD cable trench concrete casting
+[Plant Substation(SIEMENS)] Half fire wall concrete casting (Power transformer area)
+[Plant Substation(SIEMENS)] STATCOM foundation rebar binding
+[Transmission Line (SRICHONLATHORN)] Concrete foundation casting
+[Transmission Line (SRICHONLATHORN)] Foundation installation
+[Transmission Line (SRICHONLATHORN)] Column installation
+[Transmission Line (SRICHONLATHORN)] Equipment and overhead installation
+[Transmission Line (SRICHONLATHORN)] Cable pulling</t>
         </is>
       </c>
     </row>

</xml_diff>